<commit_message>
CBA update: work and leisure time shares calculated again with correct division of trip types
</commit_message>
<xml_diff>
--- a/Scripts/CBA_kehikko.xlsx
+++ b/Scripts/CBA_kehikko.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="TämäTyökirja"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HajduPe\Emme_Helmet5\model-systems\helmet-model-system\Scripts\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hslfi-my.sharepoint.com/personal/petr_hajduk_hsl_fi/Documents/Helmet ideoita/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDFB1506-52E0-4803-B444-E388D90DFD0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="47" documentId="8_{B35CA5D0-B0C9-43C8-A0D8-4ED950671617}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5F9CA642-D1F2-46A3-8903-6B2BAC49DC43}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="25695" yWindow="0" windowWidth="26010" windowHeight="20985" firstSheet="2" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Yhteenveto" sheetId="1" r:id="rId1"/>
@@ -17270,13 +17270,13 @@
     </row>
     <row r="4" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="263">
-        <v>0.46600000000000003</v>
+        <v>0.42491089427065992</v>
       </c>
       <c r="C4" s="264">
-        <v>0.10299999999999999</v>
+        <v>9.2903879644533963E-2</v>
       </c>
       <c r="D4" s="265">
-        <v>0.38500000000000001</v>
+        <v>0.4017109482228714</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -17817,13 +17817,13 @@
     </row>
     <row r="4" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="263">
-        <v>0.48</v>
+        <v>0.50581190904305739</v>
       </c>
       <c r="C4" s="264">
-        <v>9.0999999999999998E-2</v>
+        <v>9.5982138594241886E-2</v>
       </c>
       <c r="D4" s="265">
-        <v>0.39100000000000001</v>
+        <v>0.38355689167496898</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -18364,13 +18364,13 @@
     </row>
     <row r="4" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="263">
-        <v>0.59299999999999997</v>
+        <v>0.53342735671064745</v>
       </c>
       <c r="C4" s="264">
-        <v>0.112</v>
+        <v>0.11082732388014423</v>
       </c>
       <c r="D4" s="265">
-        <v>0.40799999999999997</v>
+        <v>0.4141292305134584</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -18911,13 +18911,13 @@
     </row>
     <row r="4" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="263">
-        <v>0.45100000000000001</v>
+        <v>0.6114786033543812</v>
       </c>
       <c r="C4" s="264">
-        <v>0.10100000000000001</v>
+        <v>0.10778752554496075</v>
       </c>
       <c r="D4" s="265">
-        <v>0.39300000000000002</v>
+        <v>0.40031292013253905</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -19458,13 +19458,13 @@
     </row>
     <row r="4" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="263">
-        <v>0.63600000000000001</v>
+        <v>0.62831936060779381</v>
       </c>
       <c r="C4" s="264">
-        <v>0.123</v>
+        <v>0.13760094773974157</v>
       </c>
       <c r="D4" s="265">
-        <v>0.48</v>
+        <v>0.5202210117903624</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -20005,13 +20005,13 @@
     </row>
     <row r="4" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="263">
-        <v>0.501</v>
+        <v>0.62175078551802898</v>
       </c>
       <c r="C4" s="264">
-        <v>7.2999999999999995E-2</v>
+        <v>8.663059093244195E-2</v>
       </c>
       <c r="D4" s="265">
-        <v>0.28899999999999998</v>
+        <v>0.36799378554134915</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -20517,6 +20517,41 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <DokumentinTila xmlns="37b6a217-4fe1-4884-a4eb-572c5a1969c7" xsi:nil="true"/>
+    <c7e7d47415304583b97cbceafb48fc9c xmlns="37b6a217-4fe1-4884-a4eb-572c5a1969c7">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+        <TermInfo xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+          <TermName xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">Taulukko</TermName>
+          <TermId xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">71909737-5f26-44ee-a6fd-ea06d44b9a81</TermId>
+        </TermInfo>
+      </Terms>
+    </c7e7d47415304583b97cbceafb48fc9c>
+    <TyoryhmanNimi xmlns="37b6a217-4fe1-4884-a4eb-572c5a1969c7">MAL 2019 - Kustannushyötyanalyysi</TyoryhmanNimi>
+    <gbd2c824d606482d8ac0e417e142bc2f xmlns="37b6a217-4fe1-4884-a4eb-572c5a1969c7">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </gbd2c824d606482d8ac0e417e142bc2f>
+    <lf2a24d45b2949218b95d66f1d0b33a8 xmlns="37b6a217-4fe1-4884-a4eb-572c5a1969c7">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lf2a24d45b2949218b95d66f1d0b33a8>
+    <TaxCatchAll xmlns="8dde8a50-f86d-46ca-ae54-a219d58ab0f1">
+      <Value>2</Value>
+    </TaxCatchAll>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Työryhmän dokumentti" ma:contentTypeID="0x0101005AF0DAC6D8B8D046AA97775D0EA0A52C00597B3796DB9FF548BDFCB0DE8988F274" ma:contentTypeVersion="18" ma:contentTypeDescription="" ma:contentTypeScope="" ma:versionID="52111fa3d5fab8e48da38903eaacec4d">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="37b6a217-4fe1-4884-a4eb-572c5a1969c7" xmlns:ns3="8dde8a50-f86d-46ca-ae54-a219d58ab0f1" xmlns:ns4="4468c9de-2a81-4c06-bf49-e269715ababb" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="eb907d030b2bbafc68088718dbf26d11" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="37b6a217-4fe1-4884-a4eb-572c5a1969c7"/>
@@ -20751,57 +20786,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <DokumentinTila xmlns="37b6a217-4fe1-4884-a4eb-572c5a1969c7" xsi:nil="true"/>
-    <c7e7d47415304583b97cbceafb48fc9c xmlns="37b6a217-4fe1-4884-a4eb-572c5a1969c7">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-        <TermInfo xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-          <TermName xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">Taulukko</TermName>
-          <TermId xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">71909737-5f26-44ee-a6fd-ea06d44b9a81</TermId>
-        </TermInfo>
-      </Terms>
-    </c7e7d47415304583b97cbceafb48fc9c>
-    <TyoryhmanNimi xmlns="37b6a217-4fe1-4884-a4eb-572c5a1969c7">MAL 2019 - Kustannushyötyanalyysi</TyoryhmanNimi>
-    <gbd2c824d606482d8ac0e417e142bc2f xmlns="37b6a217-4fe1-4884-a4eb-572c5a1969c7">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </gbd2c824d606482d8ac0e417e142bc2f>
-    <lf2a24d45b2949218b95d66f1d0b33a8 xmlns="37b6a217-4fe1-4884-a4eb-572c5a1969c7">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lf2a24d45b2949218b95d66f1d0b33a8>
-    <TaxCatchAll xmlns="8dde8a50-f86d-46ca-ae54-a219d58ab0f1">
-      <Value>2</Value>
-    </TaxCatchAll>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6F2FF8B0-9374-422E-84FD-E99C507D087D}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{86B210B1-4CBB-440B-90E0-17B0C211902F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="37b6a217-4fe1-4884-a4eb-572c5a1969c7"/>
-    <ds:schemaRef ds:uri="8dde8a50-f86d-46ca-ae54-a219d58ab0f1"/>
-    <ds:schemaRef ds:uri="4468c9de-2a81-4c06-bf49-e269715ababb"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -20825,9 +20813,21 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{86B210B1-4CBB-440B-90E0-17B0C211902F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6F2FF8B0-9374-422E-84FD-E99C507D087D}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="37b6a217-4fe1-4884-a4eb-572c5a1969c7"/>
+    <ds:schemaRef ds:uri="8dde8a50-f86d-46ca-ae54-a219d58ab0f1"/>
+    <ds:schemaRef ds:uri="4468c9de-2a81-4c06-bf49-e269715ababb"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
CBA updated to include new expansion factors for HELMET 5.1
</commit_message>
<xml_diff>
--- a/Scripts/CBA_kehikko.xlsx
+++ b/Scripts/CBA_kehikko.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr codeName="TämäTyökirja"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\helmet_50\model-systems\new_branch\Scripts\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HajduPe\Emme_Helmet5\model-systems\helmet-model-system\Scripts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{965B3989-6A13-4067-A10F-BF3CD92FABA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EA1A3AE-9B41-49EE-97A3-3EE50D8922E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" firstSheet="1" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Yhteenveto" sheetId="1" r:id="rId1"/>
@@ -3214,13 +3214,13 @@
     </row>
     <row r="4" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="253">
-        <v>0.501</v>
+        <v>0.62175078551802898</v>
       </c>
       <c r="C4" s="254">
-        <v>7.2999999999999995E-2</v>
+        <v>8.663059093244195E-2</v>
       </c>
       <c r="D4" s="255">
-        <v>0.28899999999999998</v>
+        <v>0.36799378554134915</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -30691,13 +30691,13 @@
     </row>
     <row r="4" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="253">
-        <v>0.48</v>
+        <v>0.50581190904305739</v>
       </c>
       <c r="C4" s="254">
-        <v>9.0999999999999998E-2</v>
+        <v>9.5982138594241886E-2</v>
       </c>
       <c r="D4" s="255">
-        <v>0.39100000000000001</v>
+        <v>0.38355689167496898</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -31242,13 +31242,13 @@
     </row>
     <row r="4" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="253">
-        <v>0.59299999999999997</v>
+        <v>0.53342735671064745</v>
       </c>
       <c r="C4" s="254">
-        <v>0.112</v>
+        <v>0.11082732388014423</v>
       </c>
       <c r="D4" s="255">
-        <v>0.40799999999999997</v>
+        <v>0.4141292305134584</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -31793,13 +31793,13 @@
     </row>
     <row r="4" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="253">
-        <v>0.45100000000000001</v>
+        <v>0.6114786033543812</v>
       </c>
       <c r="C4" s="254">
-        <v>0.10100000000000001</v>
+        <v>0.10778752554496075</v>
       </c>
       <c r="D4" s="255">
-        <v>0.39300000000000002</v>
+        <v>0.40031292013253905</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -32344,13 +32344,13 @@
     </row>
     <row r="4" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="253">
-        <v>0.63600000000000001</v>
+        <v>0.62831936060779381</v>
       </c>
       <c r="C4" s="254">
-        <v>0.123</v>
+        <v>0.13760094773974157</v>
       </c>
       <c r="D4" s="255">
-        <v>0.48</v>
+        <v>0.5202210117903624</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -32860,32 +32860,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <DokumentinTila xmlns="37b6a217-4fe1-4884-a4eb-572c5a1969c7" xsi:nil="true"/>
-    <c7e7d47415304583b97cbceafb48fc9c xmlns="37b6a217-4fe1-4884-a4eb-572c5a1969c7">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-        <TermInfo xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-          <TermName xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">Taulukko</TermName>
-          <TermId xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">71909737-5f26-44ee-a6fd-ea06d44b9a81</TermId>
-        </TermInfo>
-      </Terms>
-    </c7e7d47415304583b97cbceafb48fc9c>
-    <TyoryhmanNimi xmlns="37b6a217-4fe1-4884-a4eb-572c5a1969c7">MAL 2019 - Kustannushyötyanalyysi</TyoryhmanNimi>
-    <gbd2c824d606482d8ac0e417e142bc2f xmlns="37b6a217-4fe1-4884-a4eb-572c5a1969c7">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </gbd2c824d606482d8ac0e417e142bc2f>
-    <lf2a24d45b2949218b95d66f1d0b33a8 xmlns="37b6a217-4fe1-4884-a4eb-572c5a1969c7">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lf2a24d45b2949218b95d66f1d0b33a8>
-    <TaxCatchAll xmlns="8dde8a50-f86d-46ca-ae54-a219d58ab0f1">
-      <Value>2</Value>
-    </TaxCatchAll>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -32894,7 +32868,7 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Työryhmän dokumentti" ma:contentTypeID="0x0101005AF0DAC6D8B8D046AA97775D0EA0A52C00597B3796DB9FF548BDFCB0DE8988F274" ma:contentTypeVersion="18" ma:contentTypeDescription="" ma:contentTypeScope="" ma:versionID="52111fa3d5fab8e48da38903eaacec4d">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="37b6a217-4fe1-4884-a4eb-572c5a1969c7" xmlns:ns3="8dde8a50-f86d-46ca-ae54-a219d58ab0f1" xmlns:ns4="4468c9de-2a81-4c06-bf49-e269715ababb" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="eb907d030b2bbafc68088718dbf26d11" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="37b6a217-4fe1-4884-a4eb-572c5a1969c7"/>
@@ -33129,25 +33103,33 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EFD55EAC-37BA-4509-9765-6FB27F6E2583}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="37b6a217-4fe1-4884-a4eb-572c5a1969c7"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="4468c9de-2a81-4c06-bf49-e269715ababb"/>
-    <ds:schemaRef ds:uri="8dde8a50-f86d-46ca-ae54-a219d58ab0f1"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <DokumentinTila xmlns="37b6a217-4fe1-4884-a4eb-572c5a1969c7" xsi:nil="true"/>
+    <c7e7d47415304583b97cbceafb48fc9c xmlns="37b6a217-4fe1-4884-a4eb-572c5a1969c7">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+        <TermInfo xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+          <TermName xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">Taulukko</TermName>
+          <TermId xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">71909737-5f26-44ee-a6fd-ea06d44b9a81</TermId>
+        </TermInfo>
+      </Terms>
+    </c7e7d47415304583b97cbceafb48fc9c>
+    <TyoryhmanNimi xmlns="37b6a217-4fe1-4884-a4eb-572c5a1969c7">MAL 2019 - Kustannushyötyanalyysi</TyoryhmanNimi>
+    <gbd2c824d606482d8ac0e417e142bc2f xmlns="37b6a217-4fe1-4884-a4eb-572c5a1969c7">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </gbd2c824d606482d8ac0e417e142bc2f>
+    <lf2a24d45b2949218b95d66f1d0b33a8 xmlns="37b6a217-4fe1-4884-a4eb-572c5a1969c7">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lf2a24d45b2949218b95d66f1d0b33a8>
+    <TaxCatchAll xmlns="8dde8a50-f86d-46ca-ae54-a219d58ab0f1">
+      <Value>2</Value>
+    </TaxCatchAll>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{86B210B1-4CBB-440B-90E0-17B0C211902F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
@@ -33155,7 +33137,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6F2FF8B0-9374-422E-84FD-E99C507D087D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -33173,4 +33155,22 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EFD55EAC-37BA-4509-9765-6FB27F6E2583}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="37b6a217-4fe1-4884-a4eb-572c5a1969c7"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="4468c9de-2a81-4c06-bf49-e269715ababb"/>
+    <ds:schemaRef ds:uri="8dde8a50-f86d-46ca-ae54-a219d58ab0f1"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
car_work trips were somehow not updated in the previous commit
</commit_message>
<xml_diff>
--- a/Scripts/CBA_kehikko.xlsx
+++ b/Scripts/CBA_kehikko.xlsx
@@ -8,24 +8,24 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HajduPe\Emme_Helmet5\model-systems\helmet-model-system\Scripts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EA1A3AE-9B41-49EE-97A3-3EE50D8922E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{596F3A89-9672-4B4B-ACA5-BC2E098B355B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" firstSheet="1" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="25695" yWindow="0" windowWidth="26010" windowHeight="20985" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Yhteenveto" sheetId="1" r:id="rId1"/>
     <sheet name="Diskonttaus" sheetId="2" r:id="rId2"/>
     <sheet name="Liukuvat yksikkoarvot" sheetId="17" r:id="rId3"/>
     <sheet name="Kayttajahyodyt" sheetId="3" r:id="rId4"/>
-    <sheet name="ha_tyo" sheetId="8" state="hidden" r:id="rId5"/>
-    <sheet name="ha_muu" sheetId="11" state="hidden" r:id="rId6"/>
-    <sheet name="jl_tyo" sheetId="10" state="hidden" r:id="rId7"/>
-    <sheet name="jl_muu" sheetId="12" state="hidden" r:id="rId8"/>
-    <sheet name="pp_tyo" sheetId="13" state="hidden" r:id="rId9"/>
-    <sheet name="pp_muu" sheetId="14" state="hidden" r:id="rId10"/>
-    <sheet name="ka" sheetId="15" state="hidden" r:id="rId11"/>
-    <sheet name="yhd" sheetId="16" state="hidden" r:id="rId12"/>
-    <sheet name="pa" sheetId="9" state="hidden" r:id="rId13"/>
+    <sheet name="ha_tyo" sheetId="8" r:id="rId5"/>
+    <sheet name="ha_muu" sheetId="11" r:id="rId6"/>
+    <sheet name="jl_tyo" sheetId="10" r:id="rId7"/>
+    <sheet name="jl_muu" sheetId="12" r:id="rId8"/>
+    <sheet name="pp_tyo" sheetId="13" r:id="rId9"/>
+    <sheet name="pp_muu" sheetId="14" r:id="rId10"/>
+    <sheet name="ka" sheetId="15" r:id="rId11"/>
+    <sheet name="yhd" sheetId="16" r:id="rId12"/>
+    <sheet name="pa" sheetId="9" r:id="rId13"/>
     <sheet name="Tuottajahyodyt" sheetId="4" r:id="rId14"/>
     <sheet name="Ulkoisvaikutukset" sheetId="5" r:id="rId15"/>
     <sheet name="Julkistaloudelliset" sheetId="6" r:id="rId16"/>
@@ -30140,13 +30140,13 @@
     </row>
     <row r="4" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="253">
-        <v>0.46600000000000003</v>
+        <v>0.42491089427065992</v>
       </c>
       <c r="C4" s="254">
-        <v>0.10299999999999999</v>
+        <v>9.2903879644533963E-2</v>
       </c>
       <c r="D4" s="255">
-        <v>0.38500000000000001</v>
+        <v>0.4017109482228714</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -32869,6 +32869,32 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <DokumentinTila xmlns="37b6a217-4fe1-4884-a4eb-572c5a1969c7" xsi:nil="true"/>
+    <c7e7d47415304583b97cbceafb48fc9c xmlns="37b6a217-4fe1-4884-a4eb-572c5a1969c7">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+        <TermInfo xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+          <TermName xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">Taulukko</TermName>
+          <TermId xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">71909737-5f26-44ee-a6fd-ea06d44b9a81</TermId>
+        </TermInfo>
+      </Terms>
+    </c7e7d47415304583b97cbceafb48fc9c>
+    <TyoryhmanNimi xmlns="37b6a217-4fe1-4884-a4eb-572c5a1969c7">MAL 2019 - Kustannushyötyanalyysi</TyoryhmanNimi>
+    <gbd2c824d606482d8ac0e417e142bc2f xmlns="37b6a217-4fe1-4884-a4eb-572c5a1969c7">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </gbd2c824d606482d8ac0e417e142bc2f>
+    <lf2a24d45b2949218b95d66f1d0b33a8 xmlns="37b6a217-4fe1-4884-a4eb-572c5a1969c7">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lf2a24d45b2949218b95d66f1d0b33a8>
+    <TaxCatchAll xmlns="8dde8a50-f86d-46ca-ae54-a219d58ab0f1">
+      <Value>2</Value>
+    </TaxCatchAll>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Työryhmän dokumentti" ma:contentTypeID="0x0101005AF0DAC6D8B8D046AA97775D0EA0A52C00597B3796DB9FF548BDFCB0DE8988F274" ma:contentTypeVersion="18" ma:contentTypeDescription="" ma:contentTypeScope="" ma:versionID="52111fa3d5fab8e48da38903eaacec4d">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="37b6a217-4fe1-4884-a4eb-572c5a1969c7" xmlns:ns3="8dde8a50-f86d-46ca-ae54-a219d58ab0f1" xmlns:ns4="4468c9de-2a81-4c06-bf49-e269715ababb" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="eb907d030b2bbafc68088718dbf26d11" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="37b6a217-4fe1-4884-a4eb-572c5a1969c7"/>
@@ -33103,32 +33129,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <DokumentinTila xmlns="37b6a217-4fe1-4884-a4eb-572c5a1969c7" xsi:nil="true"/>
-    <c7e7d47415304583b97cbceafb48fc9c xmlns="37b6a217-4fe1-4884-a4eb-572c5a1969c7">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-        <TermInfo xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-          <TermName xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">Taulukko</TermName>
-          <TermId xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">71909737-5f26-44ee-a6fd-ea06d44b9a81</TermId>
-        </TermInfo>
-      </Terms>
-    </c7e7d47415304583b97cbceafb48fc9c>
-    <TyoryhmanNimi xmlns="37b6a217-4fe1-4884-a4eb-572c5a1969c7">MAL 2019 - Kustannushyötyanalyysi</TyoryhmanNimi>
-    <gbd2c824d606482d8ac0e417e142bc2f xmlns="37b6a217-4fe1-4884-a4eb-572c5a1969c7">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </gbd2c824d606482d8ac0e417e142bc2f>
-    <lf2a24d45b2949218b95d66f1d0b33a8 xmlns="37b6a217-4fe1-4884-a4eb-572c5a1969c7">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lf2a24d45b2949218b95d66f1d0b33a8>
-    <TaxCatchAll xmlns="8dde8a50-f86d-46ca-ae54-a219d58ab0f1">
-      <Value>2</Value>
-    </TaxCatchAll>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{86B210B1-4CBB-440B-90E0-17B0C211902F}">
   <ds:schemaRefs>
@@ -33138,6 +33138,24 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EFD55EAC-37BA-4509-9765-6FB27F6E2583}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="37b6a217-4fe1-4884-a4eb-572c5a1969c7"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="4468c9de-2a81-4c06-bf49-e269715ababb"/>
+    <ds:schemaRef ds:uri="8dde8a50-f86d-46ca-ae54-a219d58ab0f1"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6F2FF8B0-9374-422E-84FD-E99C507D087D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -33155,22 +33173,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EFD55EAC-37BA-4509-9765-6FB27F6E2583}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="37b6a217-4fe1-4884-a4eb-572c5a1969c7"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="4468c9de-2a81-4c06-bf49-e269715ababb"/>
-    <ds:schemaRef ds:uri="8dde8a50-f86d-46ca-ae54-a219d58ab0f1"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Forgot to hide the extra sheets
</commit_message>
<xml_diff>
--- a/Scripts/CBA_kehikko.xlsx
+++ b/Scripts/CBA_kehikko.xlsx
@@ -8,24 +8,24 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HajduPe\Emme_Helmet5\model-systems\helmet-model-system\Scripts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{596F3A89-9672-4B4B-ACA5-BC2E098B355B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77AA4EED-586F-4554-AC0A-A3F9FFBE805C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25695" yWindow="0" windowWidth="26010" windowHeight="20985" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Yhteenveto" sheetId="1" r:id="rId1"/>
     <sheet name="Diskonttaus" sheetId="2" r:id="rId2"/>
     <sheet name="Liukuvat yksikkoarvot" sheetId="17" r:id="rId3"/>
     <sheet name="Kayttajahyodyt" sheetId="3" r:id="rId4"/>
-    <sheet name="ha_tyo" sheetId="8" r:id="rId5"/>
-    <sheet name="ha_muu" sheetId="11" r:id="rId6"/>
-    <sheet name="jl_tyo" sheetId="10" r:id="rId7"/>
-    <sheet name="jl_muu" sheetId="12" r:id="rId8"/>
-    <sheet name="pp_tyo" sheetId="13" r:id="rId9"/>
-    <sheet name="pp_muu" sheetId="14" r:id="rId10"/>
-    <sheet name="ka" sheetId="15" r:id="rId11"/>
-    <sheet name="yhd" sheetId="16" r:id="rId12"/>
-    <sheet name="pa" sheetId="9" r:id="rId13"/>
+    <sheet name="ha_tyo" sheetId="8" state="hidden" r:id="rId5"/>
+    <sheet name="ha_muu" sheetId="11" state="hidden" r:id="rId6"/>
+    <sheet name="jl_tyo" sheetId="10" state="hidden" r:id="rId7"/>
+    <sheet name="jl_muu" sheetId="12" state="hidden" r:id="rId8"/>
+    <sheet name="pp_tyo" sheetId="13" state="hidden" r:id="rId9"/>
+    <sheet name="pp_muu" sheetId="14" state="hidden" r:id="rId10"/>
+    <sheet name="ka" sheetId="15" state="hidden" r:id="rId11"/>
+    <sheet name="yhd" sheetId="16" state="hidden" r:id="rId12"/>
+    <sheet name="pa" sheetId="9" state="hidden" r:id="rId13"/>
     <sheet name="Tuottajahyodyt" sheetId="4" r:id="rId14"/>
     <sheet name="Ulkoisvaikutukset" sheetId="5" r:id="rId15"/>
     <sheet name="Julkistaloudelliset" sheetId="6" r:id="rId16"/>
@@ -32869,32 +32869,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <DokumentinTila xmlns="37b6a217-4fe1-4884-a4eb-572c5a1969c7" xsi:nil="true"/>
-    <c7e7d47415304583b97cbceafb48fc9c xmlns="37b6a217-4fe1-4884-a4eb-572c5a1969c7">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-        <TermInfo xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-          <TermName xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">Taulukko</TermName>
-          <TermId xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">71909737-5f26-44ee-a6fd-ea06d44b9a81</TermId>
-        </TermInfo>
-      </Terms>
-    </c7e7d47415304583b97cbceafb48fc9c>
-    <TyoryhmanNimi xmlns="37b6a217-4fe1-4884-a4eb-572c5a1969c7">MAL 2019 - Kustannushyötyanalyysi</TyoryhmanNimi>
-    <gbd2c824d606482d8ac0e417e142bc2f xmlns="37b6a217-4fe1-4884-a4eb-572c5a1969c7">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </gbd2c824d606482d8ac0e417e142bc2f>
-    <lf2a24d45b2949218b95d66f1d0b33a8 xmlns="37b6a217-4fe1-4884-a4eb-572c5a1969c7">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lf2a24d45b2949218b95d66f1d0b33a8>
-    <TaxCatchAll xmlns="8dde8a50-f86d-46ca-ae54-a219d58ab0f1">
-      <Value>2</Value>
-    </TaxCatchAll>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Työryhmän dokumentti" ma:contentTypeID="0x0101005AF0DAC6D8B8D046AA97775D0EA0A52C00597B3796DB9FF548BDFCB0DE8988F274" ma:contentTypeVersion="18" ma:contentTypeDescription="" ma:contentTypeScope="" ma:versionID="52111fa3d5fab8e48da38903eaacec4d">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="37b6a217-4fe1-4884-a4eb-572c5a1969c7" xmlns:ns3="8dde8a50-f86d-46ca-ae54-a219d58ab0f1" xmlns:ns4="4468c9de-2a81-4c06-bf49-e269715ababb" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="eb907d030b2bbafc68088718dbf26d11" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="37b6a217-4fe1-4884-a4eb-572c5a1969c7"/>
@@ -33129,6 +33103,32 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <DokumentinTila xmlns="37b6a217-4fe1-4884-a4eb-572c5a1969c7" xsi:nil="true"/>
+    <c7e7d47415304583b97cbceafb48fc9c xmlns="37b6a217-4fe1-4884-a4eb-572c5a1969c7">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+        <TermInfo xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+          <TermName xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">Taulukko</TermName>
+          <TermId xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">71909737-5f26-44ee-a6fd-ea06d44b9a81</TermId>
+        </TermInfo>
+      </Terms>
+    </c7e7d47415304583b97cbceafb48fc9c>
+    <TyoryhmanNimi xmlns="37b6a217-4fe1-4884-a4eb-572c5a1969c7">MAL 2019 - Kustannushyötyanalyysi</TyoryhmanNimi>
+    <gbd2c824d606482d8ac0e417e142bc2f xmlns="37b6a217-4fe1-4884-a4eb-572c5a1969c7">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </gbd2c824d606482d8ac0e417e142bc2f>
+    <lf2a24d45b2949218b95d66f1d0b33a8 xmlns="37b6a217-4fe1-4884-a4eb-572c5a1969c7">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lf2a24d45b2949218b95d66f1d0b33a8>
+    <TaxCatchAll xmlns="8dde8a50-f86d-46ca-ae54-a219d58ab0f1">
+      <Value>2</Value>
+    </TaxCatchAll>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{86B210B1-4CBB-440B-90E0-17B0C211902F}">
   <ds:schemaRefs>
@@ -33138,24 +33138,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EFD55EAC-37BA-4509-9765-6FB27F6E2583}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="37b6a217-4fe1-4884-a4eb-572c5a1969c7"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="4468c9de-2a81-4c06-bf49-e269715ababb"/>
-    <ds:schemaRef ds:uri="8dde8a50-f86d-46ca-ae54-a219d58ab0f1"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6F2FF8B0-9374-422E-84FD-E99C507D087D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -33173,4 +33155,22 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EFD55EAC-37BA-4509-9765-6FB27F6E2583}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="37b6a217-4fe1-4884-a4eb-572c5a1969c7"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="4468c9de-2a81-4c06-bf49-e269715ababb"/>
+    <ds:schemaRef ds:uri="8dde8a50-f86d-46ca-ae54-a219d58ab0f1"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>